<commit_message>
roadmap: add subtasks 2.7.i-m (gold standard corrections, prompt design, rationale)
2.7.i — Gold standard v2 corrections (Failure 3 + 4) [completed]
2.7.j — Pass 1 strict prompt with corrected OUTPUT GOAL [completed]
2.7.k — Lessons Learned rationale doc [completed]
2.7.l — Pass 2 Editorial Diagnostic prompt [next]
2.7.m — Pass 3 Synthesis Engine prompt [next]

Markdown companion regenerated from xlsx.
</commit_message>
<xml_diff>
--- a/docs/RevisionGrade_Roadmap_UPDATED.xlsx
+++ b/docs/RevisionGrade_Roadmap_UPDATED.xlsx
@@ -1449,7 +1449,6 @@
         </is>
       </c>
     </row>
-    <row r="7"/>
     <row r="8" ht="14.25" customHeight="1" s="96">
       <c r="A8" s="95" t="inlineStr">
         <is>
@@ -1457,7 +1456,6 @@
         </is>
       </c>
     </row>
-    <row r="9"/>
     <row r="10" ht="14.25" customHeight="1" s="96">
       <c r="A10" s="95" t="inlineStr">
         <is>
@@ -1500,7 +1498,6 @@
         </is>
       </c>
     </row>
-    <row r="16"/>
     <row r="17" ht="14.25" customHeight="1" s="96">
       <c r="A17" s="95" t="inlineStr">
         <is>
@@ -1536,7 +1533,6 @@
         </is>
       </c>
     </row>
-    <row r="22"/>
     <row r="23" ht="14.25" customHeight="1" s="96">
       <c r="A23" s="95" t="inlineStr">
         <is>
@@ -1586,7 +1582,6 @@
         </is>
       </c>
     </row>
-    <row r="30"/>
     <row r="31" ht="14.25" customHeight="1" s="96">
       <c r="A31" s="95" t="inlineStr">
         <is>
@@ -5984,7 +5979,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="0"/>
   </sheetPr>
-  <dimension ref="A1:T40"/>
+  <dimension ref="A1:T45"/>
   <sheetFormatPr baseColWidth="8" defaultColWidth="8.6796875" defaultRowHeight="14.25" customHeight="1" zeroHeight="0" outlineLevelRow="0"/>
   <cols>
     <col width="18" customWidth="1" style="95" min="1" max="1"/>
@@ -7792,6 +7787,256 @@
       <c r="J40" s="190" t="inlineStr">
         <is>
           <t>Updated prompt files (v2), runs/run-002/ directory, PHASE_2_7_REAL_RUN_01.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" t="n">
+        <v>0</v>
+      </c>
+      <c r="B41" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="C41" t="inlineStr">
+        <is>
+          <t>Calibration Files</t>
+        </is>
+      </c>
+      <c r="D41" t="inlineStr">
+        <is>
+          <t>2.7.i</t>
+        </is>
+      </c>
+      <c r="E41" t="inlineStr">
+        <is>
+          <t>Gold standard v2 corrections — Failure 3 (authority signaling) + Failure 4 (cross-chapter causality)</t>
+        </is>
+      </c>
+      <c r="F41" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="G41" t="inlineStr">
+        <is>
+          <t>calibration/</t>
+        </is>
+      </c>
+      <c r="H41" t="inlineStr">
+        <is>
+          <t>Failure 4 correctly identifies causality as earned but under-signaled. Failure 3 diagnoses boundary signaling, not chaos.</t>
+        </is>
+      </c>
+      <c r="I41" t="inlineStr">
+        <is>
+          <t>Author review + novel text verification (Brutus/driftwood I:2.12 → Realm I:3.5 → barrier I:4)</t>
+        </is>
+      </c>
+      <c r="J41" t="inlineStr">
+        <is>
+          <t>calibration/dominatus-i4-revisiongrade-gold-standard.md (v2 corrected). Commit: 30c9336</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" t="n">
+        <v>0</v>
+      </c>
+      <c r="B42" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="C42" t="inlineStr">
+        <is>
+          <t>Prompt Design</t>
+        </is>
+      </c>
+      <c r="D42" t="inlineStr">
+        <is>
+          <t>2.7.j</t>
+        </is>
+      </c>
+      <c r="E42" t="inlineStr">
+        <is>
+          <t>Pass 1 Structural Diagnostic prompt — strict mode, layer-isolated, corrected OUTPUT GOAL (MD-2/3/4/5 only)</t>
+        </is>
+      </c>
+      <c r="F42" t="inlineStr">
+        <is>
+          <t>Prompt</t>
+        </is>
+      </c>
+      <c r="G42" t="inlineStr">
+        <is>
+          <t>prompts/</t>
+        </is>
+      </c>
+      <c r="H42" t="inlineStr">
+        <is>
+          <t>Forced eval order, mandatory taxonomy, anti-pattern enforcement, MD-1/MD-6 excluded (Pass 2 scope)</t>
+        </is>
+      </c>
+      <c r="I42" t="inlineStr">
+        <is>
+          <t>Layer isolation check: prompt does not reference expression-level items. Checklist alignment verified.</t>
+        </is>
+      </c>
+      <c r="J42" t="inlineStr">
+        <is>
+          <t>prompts/pass-1-structural-diagnostic.md. Commit: a0f9d36</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" t="n">
+        <v>0</v>
+      </c>
+      <c r="B43" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="C43" t="inlineStr">
+        <is>
+          <t>Governance</t>
+        </is>
+      </c>
+      <c r="D43" t="inlineStr">
+        <is>
+          <t>2.7.k</t>
+        </is>
+      </c>
+      <c r="E43" t="inlineStr">
+        <is>
+          <t>Lessons Learned — Pass 1 design rationale (4 primitives, rejected alternatives, sufficiency claim)</t>
+        </is>
+      </c>
+      <c r="F43" t="inlineStr">
+        <is>
+          <t>Doc</t>
+        </is>
+      </c>
+      <c r="G43" t="inlineStr">
+        <is>
+          <t>docs/rationale/</t>
+        </is>
+      </c>
+      <c r="H43" t="inlineStr">
+        <is>
+          <t>Covers: why these 4, why not theme/character/pacing/prose/WAVE/scene-entry, checklist alignment, risks, mitigations</t>
+        </is>
+      </c>
+      <c r="I43" t="inlineStr">
+        <is>
+          <t>Rationale doc stands as independent justification. Canon/rationale separation enforced.</t>
+        </is>
+      </c>
+      <c r="J43" t="inlineStr">
+        <is>
+          <t>docs/rationale/LESSONS_LEARNED_PHASE_2_7.md. Commit: a0f9d36</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" t="n">
+        <v>0</v>
+      </c>
+      <c r="B44" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="C44" t="inlineStr">
+        <is>
+          <t>Prompt Design</t>
+        </is>
+      </c>
+      <c r="D44" t="inlineStr">
+        <is>
+          <t>2.7.l</t>
+        </is>
+      </c>
+      <c r="E44" t="inlineStr">
+        <is>
+          <t>Pass 2 Editorial Diagnostic prompt — expression layer (WAVE + 13 Criteria, MD-1/MD-6 scope)</t>
+        </is>
+      </c>
+      <c r="F44" t="inlineStr">
+        <is>
+          <t>Prompt</t>
+        </is>
+      </c>
+      <c r="G44" t="inlineStr">
+        <is>
+          <t>prompts/</t>
+        </is>
+      </c>
+      <c r="H44" t="inlineStr">
+        <is>
+          <t>Detects thematic overstatement, metaphor conflicts, echo chains, non-observable language, personification density. Scores against MD-1, MD-6, SD-1 through SD-6.</t>
+        </is>
+      </c>
+      <c r="I44" t="inlineStr">
+        <is>
+          <t>Layer isolation: prompt does not duplicate Pass 1 structural items. Checklist alignment verified.</t>
+        </is>
+      </c>
+      <c r="J44" t="inlineStr">
+        <is>
+          <t>prompts/pass-2-editorial-diagnostic.md</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" t="n">
+        <v>0</v>
+      </c>
+      <c r="B45" t="inlineStr">
+        <is>
+          <t>2.7</t>
+        </is>
+      </c>
+      <c r="C45" t="inlineStr">
+        <is>
+          <t>Prompt Design</t>
+        </is>
+      </c>
+      <c r="D45" t="inlineStr">
+        <is>
+          <t>2.7.m</t>
+        </is>
+      </c>
+      <c r="E45" t="inlineStr">
+        <is>
+          <t>Pass 3 Synthesis Engine prompt — priority ordering, cross-layer integration, execution plan</t>
+        </is>
+      </c>
+      <c r="F45" t="inlineStr">
+        <is>
+          <t>Prompt</t>
+        </is>
+      </c>
+      <c r="G45" t="inlineStr">
+        <is>
+          <t>prompts/</t>
+        </is>
+      </c>
+      <c r="H45" t="inlineStr">
+        <is>
+          <t>Ranks failures (architecture → line-level), explains interactions, defines fix sequence. Scores against SI-1 through SI-4.</t>
+        </is>
+      </c>
+      <c r="I45" t="inlineStr">
+        <is>
+          <t>Output produces actionable execution plan with structural issues ranked above expression issues.</t>
+        </is>
+      </c>
+      <c r="J45" t="inlineStr">
+        <is>
+          <t>prompts/pass-3-synthesis-engine.md</t>
         </is>
       </c>
     </row>

</xml_diff>